<commit_message>
Fix unbounded models and solver crashes, update test script
</commit_message>
<xml_diff>
--- a/src/strap/waste_management/Data for model_Scenarios.xlsx
+++ b/src/strap/waste_management/Data for model_Scenarios.xlsx
@@ -6424,7 +6424,7 @@
         <v>0.1795217098507607</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>0.08668835839130781</v>
+        <v>0.08668835839130783</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>4842268.133639095</v>
@@ -6453,7 +6453,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>203322812427.7125</v>
+        <v>203322812427.7126</v>
       </c>
       <c r="E3" t="n">
         <v>2642745.600000001</v>
@@ -6486,7 +6486,7 @@
         <v>0.08667031655450493</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>4841217.409068096</v>
+        <v>4841217.409068097</v>
       </c>
       <c r="P3" s="4" t="n">
         <v>1649512.153</v>
@@ -6518,7 +6518,7 @@
         <v>2536588.8</v>
       </c>
       <c r="F4" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -6536,16 +6536,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.1543060585272763</v>
+        <v>0.1543060585272762</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0.07448869386639052</v>
+        <v>0.07448869386639051</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4159676.202236705</v>
+        <v>4159676.202236703</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>1376265.6805</v>
@@ -6577,7 +6577,7 @@
         <v>2637158.4</v>
       </c>
       <c r="F5" t="n">
-        <v>4881.717512393886</v>
+        <v>4881.717512393888</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -6595,16 +6595,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>4881.717512393886</v>
+        <v>4881.717512393888</v>
       </c>
       <c r="M5" s="4" t="n">
         <v>0.1838829672485295</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.08877707982610991</v>
+        <v>0.08877707982610993</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>4959629.214836514</v>
+        <v>4959629.214836515</v>
       </c>
       <c r="P5" s="4" t="n">
         <v>1588570.236</v>
@@ -6716,13 +6716,13 @@
         <v>7133.280889431222</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.2688143651603698</v>
+        <v>0.2688143651603699</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.1300059288112211</v>
+        <v>0.1300059288112212</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>7258707.340225391</v>
+        <v>7258707.340225393</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>1894036.3775</v>
@@ -6807,7 +6807,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>201354897959.7588</v>
+        <v>201354897959.7589</v>
       </c>
       <c r="E9" t="n">
         <v>2720966.4</v>
@@ -6925,7 +6925,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37834039978.64439</v>
+        <v>37834039978.64438</v>
       </c>
       <c r="E11" t="n">
         <v>616454.4</v>
@@ -7073,7 +7073,7 @@
         <v>0.1795217098507607</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.08668835839130781</v>
+        <v>0.08668835839130783</v>
       </c>
       <c r="O13" s="4" t="n">
         <v>4842268.133639095</v>
@@ -7102,7 +7102,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>203322812427.7125</v>
+        <v>203322812427.7126</v>
       </c>
       <c r="E14" t="n">
         <v>2637158.4</v>
@@ -7135,7 +7135,7 @@
         <v>0.08667031655450493</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>4841217.409068096</v>
+        <v>4841217.409068097</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>1652358.963</v>
@@ -7167,7 +7167,7 @@
         <v>2536588.8</v>
       </c>
       <c r="F15" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -7185,16 +7185,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.1543060585272763</v>
+        <v>0.1543060585272762</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.07448869386639052</v>
+        <v>0.07448869386639051</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>4159676.202236705</v>
+        <v>4159676.202236703</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>1371700.307</v>
@@ -7226,7 +7226,7 @@
         <v>2631571.2</v>
       </c>
       <c r="F16" t="n">
-        <v>4881.717512393886</v>
+        <v>4881.717512393888</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -7244,16 +7244,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>4881.717512393886</v>
+        <v>4881.717512393888</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>0.1838829672485295</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>0.08877707982610991</v>
+        <v>0.08877707982610993</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>4959629.214836514</v>
+        <v>4959629.214836515</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>1590719.481</v>
@@ -7365,13 +7365,13 @@
         <v>7133.280889431222</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0.2688143651603698</v>
+        <v>0.2688143651603699</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>0.1300059288112211</v>
+        <v>0.1300059288112212</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>7258707.340225391</v>
+        <v>7258707.340225393</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>1893805.082</v>
@@ -7456,7 +7456,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>201354897959.7588</v>
+        <v>201354897959.7589</v>
       </c>
       <c r="E20" t="n">
         <v>2715379.2</v>
@@ -7574,7 +7574,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>38153266139.19757</v>
+        <v>38153266139.19758</v>
       </c>
       <c r="E22" t="n">
         <v>508435.2</v>
@@ -7751,7 +7751,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>37834039978.64439</v>
+        <v>37834039978.64438</v>
       </c>
       <c r="E25" t="n">
         <v>506572.8</v>

</xml_diff>

<commit_message>
Apply exact paper GWP fallback values for Gasification variants missing from Excel
</commit_message>
<xml_diff>
--- a/src/strap/waste_management/Data for model_Scenarios.xlsx
+++ b/src/strap/waste_management/Data for model_Scenarios.xlsx
@@ -6518,7 +6518,7 @@
         <v>2536588.8</v>
       </c>
       <c r="F4" t="n">
-        <v>4098.763512502048</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -6536,16 +6536,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>4098.763512502048</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.1543060585272762</v>
+        <v>0.1543060585272763</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0.07448869386639051</v>
+        <v>0.07448869386639052</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4159676.202236703</v>
+        <v>4159676.202236705</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>1376265.6805</v>
@@ -6577,7 +6577,7 @@
         <v>2637158.4</v>
       </c>
       <c r="F5" t="n">
-        <v>4881.717512393888</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -6595,16 +6595,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>4881.717512393888</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="M5" s="4" t="n">
         <v>0.1838829672485295</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.08877707982610993</v>
+        <v>0.08877707982610991</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>4959629.214836515</v>
+        <v>4959629.214836514</v>
       </c>
       <c r="P5" s="4" t="n">
         <v>1588570.236</v>
@@ -6716,13 +6716,13 @@
         <v>7133.280889431222</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.2688143651603699</v>
+        <v>0.2688143651603698</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.1300059288112212</v>
+        <v>0.1300059288112211</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>7258707.340225393</v>
+        <v>7258707.340225391</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>1894036.3775</v>
@@ -7167,7 +7167,7 @@
         <v>2536588.8</v>
       </c>
       <c r="F15" t="n">
-        <v>4098.763512502048</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -7185,16 +7185,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4098.763512502048</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.1543060585272762</v>
+        <v>0.1543060585272763</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.07448869386639051</v>
+        <v>0.07448869386639052</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>4159676.202236703</v>
+        <v>4159676.202236705</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>1371700.307</v>
@@ -7226,7 +7226,7 @@
         <v>2631571.2</v>
       </c>
       <c r="F16" t="n">
-        <v>4881.717512393888</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -7244,16 +7244,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>4881.717512393888</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>0.1838829672485295</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>0.08877707982610993</v>
+        <v>0.08877707982610991</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>4959629.214836515</v>
+        <v>4959629.214836514</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>1590719.481</v>
@@ -7365,13 +7365,13 @@
         <v>7133.280889431222</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0.2688143651603699</v>
+        <v>0.2688143651603698</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>0.1300059288112212</v>
+        <v>0.1300059288112211</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>7258707.340225393</v>
+        <v>7258707.340225391</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>1893805.082</v>
@@ -7692,7 +7692,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>38342696728.86108</v>
+        <v>38342696728.86106</v>
       </c>
       <c r="E24" t="n">
         <v>515884.8</v>
@@ -7719,10 +7719,10 @@
         <v>1142.336921530873</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>0.04303976596610721</v>
+        <v>0.0430397659661072</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>0.02077703132808372</v>
+        <v>0.02077703132808371</v>
       </c>
       <c r="O24" s="4" t="n">
         <v>1160821.53924672</v>

</xml_diff>

<commit_message>
Fix Pareto optimization scaling bug. Extract _update_excel_with_biosteam helper to ensure Pareto sweeps dynamically calculate CAPEX/OPEX based on feed size instead of using stale Excel data.
</commit_message>
<xml_diff>
--- a/src/strap/waste_management/Data for model_Scenarios.xlsx
+++ b/src/strap/waste_management/Data for model_Scenarios.xlsx
@@ -6424,7 +6424,7 @@
         <v>0.1795217098507607</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>0.08668835839130783</v>
+        <v>0.08668835839130781</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>4842268.133639095</v>
@@ -6518,7 +6518,7 @@
         <v>2536588.8</v>
       </c>
       <c r="F4" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -6536,16 +6536,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.1543060585272763</v>
+        <v>0.1543060585272762</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0.07448869386639052</v>
+        <v>0.07448869386639051</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4159676.202236705</v>
+        <v>4159676.202236703</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>1376265.6805</v>
@@ -6813,7 +6813,7 @@
         <v>2720966.4</v>
       </c>
       <c r="F9" t="n">
-        <v>4588.054944384647</v>
+        <v>4588.054944384648</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -6831,7 +6831,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>4588.054944384647</v>
+        <v>4588.054944384648</v>
       </c>
       <c r="M9" s="4" t="n">
         <v>0.1727735587845355</v>
@@ -6840,7 +6840,7 @@
         <v>0.08337812122162949</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>4658031.659165952</v>
+        <v>4658031.659165954</v>
       </c>
       <c r="P9" s="4" t="n">
         <v>1935089.606</v>
@@ -6925,7 +6925,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37834039978.64438</v>
+        <v>37834039978.64439</v>
       </c>
       <c r="E11" t="n">
         <v>616454.4</v>
@@ -6984,7 +6984,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>37359989902.81407</v>
+        <v>37359989902.81406</v>
       </c>
       <c r="E12" t="n">
         <v>586656</v>
@@ -7073,7 +7073,7 @@
         <v>0.1795217098507607</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.08668835839130783</v>
+        <v>0.08668835839130781</v>
       </c>
       <c r="O13" s="4" t="n">
         <v>4842268.133639095</v>
@@ -7167,7 +7167,7 @@
         <v>2536588.8</v>
       </c>
       <c r="F15" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -7185,16 +7185,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4098.763512502049</v>
+        <v>4098.763512502048</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.1543060585272763</v>
+        <v>0.1543060585272762</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.07448869386639052</v>
+        <v>0.07448869386639051</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>4159676.202236705</v>
+        <v>4159676.202236703</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>1371700.307</v>
@@ -7462,7 +7462,7 @@
         <v>2715379.2</v>
       </c>
       <c r="F20" t="n">
-        <v>4588.054944384647</v>
+        <v>4588.054944384648</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -7480,7 +7480,7 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>4588.054944384647</v>
+        <v>4588.054944384648</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>0.1727735587845355</v>
@@ -7489,7 +7489,7 @@
         <v>0.08337812122162949</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>4658031.659165952</v>
+        <v>4658031.659165954</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>1929337.8795</v>
@@ -7574,7 +7574,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>38153266139.19758</v>
+        <v>38153266139.19757</v>
       </c>
       <c r="E22" t="n">
         <v>508435.2</v>
@@ -7751,7 +7751,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>37834039978.64438</v>
+        <v>37834039978.64439</v>
       </c>
       <c r="E25" t="n">
         <v>506572.8</v>
@@ -7869,7 +7869,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>37359989902.81407</v>
+        <v>37359989902.81406</v>
       </c>
       <c r="E27" t="n">
         <v>492604.8</v>

</xml_diff>

<commit_message>
Add anti-hallucination rule to optimization-engineer prompt forcing tool usage
</commit_message>
<xml_diff>
--- a/src/strap/waste_management/Data for model_Scenarios.xlsx
+++ b/src/strap/waste_management/Data for model_Scenarios.xlsx
@@ -6394,13 +6394,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>202926111011.0003</v>
+        <v>665218245883.6273</v>
       </c>
       <c r="E2" t="n">
         <v>2642745.600000001</v>
       </c>
       <c r="F2" t="n">
-        <v>4765.733611442293</v>
+        <v>15666.63019162362</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -6418,16 +6418,16 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>4765.733611442293</v>
+        <v>15666.63019162362</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>0.1795217098507607</v>
+        <v>0.5901572639578164</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>0.08668835839130781</v>
+        <v>0.2849813592682811</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>4842268.133639095</v>
+        <v>15918578.82709316</v>
       </c>
       <c r="P2" s="4" t="n">
         <v>1645223.07</v>
@@ -6453,13 +6453,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>203322812427.7126</v>
+        <v>666525829696.7694</v>
       </c>
       <c r="E3" t="n">
         <v>2642745.600000001</v>
       </c>
       <c r="F3" t="n">
-        <v>4764.551000420273</v>
+        <v>15662.39951584713</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -6477,16 +6477,16 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>4764.551000420273</v>
+        <v>15662.39951584713</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.1794792887150163</v>
+        <v>0.5900049962128856</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.08667031655450493</v>
+        <v>0.2849159779978077</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>4841217.409068097</v>
+        <v>15914783.60232515</v>
       </c>
       <c r="P3" s="4" t="n">
         <v>1649512.153</v>
@@ -6512,13 +6512,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>190737625701.4836</v>
+        <v>625232124635.0183</v>
       </c>
       <c r="E4" t="n">
         <v>2536588.8</v>
       </c>
       <c r="F4" t="n">
-        <v>4098.763512502048</v>
+        <v>13455.95924340548</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -6536,16 +6536,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>4098.763512502048</v>
+        <v>13455.95924340548</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.1543060585272762</v>
+        <v>0.5065779354407081</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0.07448869386639051</v>
+        <v>0.2445439553938083</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4159676.202236703</v>
+        <v>13656016.62047045</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>1376265.6805</v>
@@ -6571,13 +6571,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>201270843091.6686</v>
+        <v>659926710982.4099</v>
       </c>
       <c r="E5" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F5" t="n">
-        <v>4881.717512393886</v>
+        <v>16057.66494595068</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -6595,16 +6595,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>4881.717512393886</v>
+        <v>16057.66494595068</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0.1838829672485295</v>
+        <v>0.6048612169850395</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.08877707982610991</v>
+        <v>0.2920240650367384</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>4959629.214836514</v>
+        <v>16314268.07134834</v>
       </c>
       <c r="P5" s="4" t="n">
         <v>1588570.236</v>
@@ -6630,13 +6630,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>203478955758.8295</v>
+        <v>666912636947.7731</v>
       </c>
       <c r="E6" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F6" t="n">
-        <v>4612.468401356314</v>
+        <v>15152.8425063876</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -6654,16 +6654,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>4612.468401356314</v>
+        <v>15152.8425063876</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>0.1737063794243002</v>
+        <v>0.570663539923043</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>0.08384112296942656</v>
+        <v>0.2754378429119639</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4684017.968013241</v>
+        <v>15388132.66903725</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>1674069.678</v>
@@ -6689,13 +6689,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>221770868690.6884</v>
+        <v>727818948453.0715</v>
       </c>
       <c r="E7" t="n">
         <v>2866233.6</v>
       </c>
       <c r="F7" t="n">
-        <v>7133.280889431222</v>
+        <v>23554.24532157016</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -6713,16 +6713,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>7133.280889431222</v>
+        <v>23554.24532157016</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.2688143651603698</v>
+        <v>0.8876410227096855</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.1300059288112211</v>
+        <v>0.4292968209774043</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>7258707.340225391</v>
+        <v>23969106.23537641</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>1894036.3775</v>
@@ -6748,13 +6748,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>206620827403.3771</v>
+        <v>677213565060.4402</v>
       </c>
       <c r="E8" t="n">
         <v>2659507.2</v>
       </c>
       <c r="F8" t="n">
-        <v>4738.270770013095</v>
+        <v>15568.81932111654</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -6772,16 +6772,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>4738.270770013095</v>
+        <v>15568.81932111654</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>0.1784311331513977</v>
+        <v>0.5862860872937612</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>0.08610805906069278</v>
+        <v>0.2829331972787671</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4810653.628441143</v>
+        <v>15806838.51117178</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>1746245.131</v>
@@ -6807,13 +6807,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>201354897959.7589</v>
+        <v>659990021842.691</v>
       </c>
       <c r="E9" t="n">
         <v>2720966.4</v>
       </c>
       <c r="F9" t="n">
-        <v>4588.054944384648</v>
+        <v>15074.54702536651</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -6831,16 +6831,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>4588.054944384648</v>
+        <v>15074.54702536651</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.1727735587845355</v>
+        <v>0.567670166528999</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>0.08337812122162949</v>
+        <v>0.273950487129699</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>4658031.659165954</v>
+        <v>15304638.88995023</v>
       </c>
       <c r="P9" s="4" t="n">
         <v>1935089.606</v>
@@ -6866,13 +6866,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>204572003174.7647</v>
+        <v>670725322277.7625</v>
       </c>
       <c r="E10" t="n">
         <v>2659507.2</v>
       </c>
       <c r="F10" t="n">
-        <v>4976.446993016055</v>
+        <v>16369.4144402207</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -6890,16 +6890,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>4976.446993016055</v>
+        <v>16369.4144402207</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0.1874216627349249</v>
+        <v>0.6165057331643525</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>0.09044810802733161</v>
+        <v>0.2975212368273295</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5053161.540511617</v>
+        <v>16621969.03072156</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>1661215.79</v>
@@ -6925,13 +6925,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37834039978.64439</v>
+        <v>89342761464.93727</v>
       </c>
       <c r="E11" t="n">
         <v>616454.4</v>
       </c>
       <c r="F11" t="n">
-        <v>1052.931970048123</v>
+        <v>2529.773421713371</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -6949,16 +6949,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1052.931970048123</v>
+        <v>2529.773421713371</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.03966801424067684</v>
+        <v>0.09530995598830956</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>0.01914863080991969</v>
+        <v>0.0460091048880134</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>1069824.932926143</v>
+        <v>2570524.007936024</v>
       </c>
       <c r="P11" s="4" t="n">
         <v>827574.618</v>
@@ -6984,13 +6984,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>37359989902.81406</v>
+        <v>88149476858.2751</v>
       </c>
       <c r="E12" t="n">
         <v>586656</v>
       </c>
       <c r="F12" t="n">
-        <v>942.4386036831032</v>
+        <v>2253.380382134857</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -7008,16 +7008,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>942.4386036831032</v>
+        <v>2253.380382134857</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>0.03552384399687809</v>
+        <v>0.08494352237307626</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>0.01717808702872767</v>
+        <v>0.04107984659757677</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>960485.5461196182</v>
+        <v>2297013.610876977</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>831337.1199999999</v>
@@ -7043,13 +7043,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>202926111011.0003</v>
+        <v>665218245883.6273</v>
       </c>
       <c r="E13" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F13" t="n">
-        <v>4765.733611442293</v>
+        <v>15666.63019162362</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -7067,16 +7067,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>4765.733611442293</v>
+        <v>15666.63019162362</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0.1795217098507607</v>
+        <v>0.5901572639578164</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.08668835839130781</v>
+        <v>0.2849813592682811</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>4842268.133639095</v>
+        <v>15918578.82709316</v>
       </c>
       <c r="P13" s="4" t="n">
         <v>1640984.363</v>
@@ -7102,13 +7102,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>203322812427.7126</v>
+        <v>666525829696.7694</v>
       </c>
       <c r="E14" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F14" t="n">
-        <v>4764.551000420273</v>
+        <v>15662.39951584713</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -7126,16 +7126,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>4764.551000420273</v>
+        <v>15662.39951584713</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>0.1794792887150163</v>
+        <v>0.5900049962128856</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>0.08667031655450493</v>
+        <v>0.2849159779978077</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>4841217.409068097</v>
+        <v>15914783.60232515</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>1652358.963</v>
@@ -7161,13 +7161,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>190737625701.4836</v>
+        <v>625232124635.0183</v>
       </c>
       <c r="E15" t="n">
         <v>2536588.8</v>
       </c>
       <c r="F15" t="n">
-        <v>4098.763512502048</v>
+        <v>13455.95924340548</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -7185,16 +7185,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4098.763512502048</v>
+        <v>13455.95924340548</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.1543060585272762</v>
+        <v>0.5065779354407081</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.07448869386639051</v>
+        <v>0.2445439553938083</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>4159676.202236703</v>
+        <v>13656016.62047045</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>1371700.307</v>
@@ -7220,13 +7220,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>201270843091.6686</v>
+        <v>659926710982.4099</v>
       </c>
       <c r="E16" t="n">
         <v>2631571.2</v>
       </c>
       <c r="F16" t="n">
-        <v>4881.717512393886</v>
+        <v>16057.66494595068</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -7244,16 +7244,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>4881.717512393886</v>
+        <v>16057.66494595068</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>0.1838829672485295</v>
+        <v>0.6048612169850395</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>0.08877707982610991</v>
+        <v>0.2920240650367384</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>4959629.214836514</v>
+        <v>16314268.07134834</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>1590719.481</v>
@@ -7279,13 +7279,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>203478955758.8295</v>
+        <v>666912636947.7731</v>
       </c>
       <c r="E17" t="n">
         <v>2631571.2</v>
       </c>
       <c r="F17" t="n">
-        <v>4612.468401356314</v>
+        <v>15152.8425063876</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -7303,16 +7303,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>4612.468401356314</v>
+        <v>15152.8425063876</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.1737063794243002</v>
+        <v>0.570663539923043</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>0.08384112296942656</v>
+        <v>0.2754378429119639</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>4684017.968013241</v>
+        <v>15388132.66903725</v>
       </c>
       <c r="P17" s="4" t="n">
         <v>1670234.7225</v>
@@ -7338,13 +7338,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>221770868690.6884</v>
+        <v>727818948453.0715</v>
       </c>
       <c r="E18" t="n">
         <v>2855059.2</v>
       </c>
       <c r="F18" t="n">
-        <v>7133.280889431222</v>
+        <v>23554.24532157016</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -7362,16 +7362,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>7133.280889431222</v>
+        <v>23554.24532157016</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0.2688143651603698</v>
+        <v>0.8876410227096855</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>0.1300059288112211</v>
+        <v>0.4292968209774043</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>7258707.340225391</v>
+        <v>23969106.23537641</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>1893805.082</v>
@@ -7397,13 +7397,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>206620827403.3771</v>
+        <v>677213565060.4402</v>
       </c>
       <c r="E19" t="n">
         <v>2653920</v>
       </c>
       <c r="F19" t="n">
-        <v>4738.270770013095</v>
+        <v>15568.81932111654</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -7421,16 +7421,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>4738.270770013095</v>
+        <v>15568.81932111654</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>0.1784311331513977</v>
+        <v>0.5862860872937612</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>0.08610805906069278</v>
+        <v>0.2829331972787671</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>4810653.628441143</v>
+        <v>15806838.51117178</v>
       </c>
       <c r="P19" s="4" t="n">
         <v>1742565.4565</v>
@@ -7456,13 +7456,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>201354897959.7589</v>
+        <v>659990021842.691</v>
       </c>
       <c r="E20" t="n">
         <v>2715379.2</v>
       </c>
       <c r="F20" t="n">
-        <v>4588.054944384648</v>
+        <v>15074.54702536651</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -7480,16 +7480,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>4588.054944384648</v>
+        <v>15074.54702536651</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>0.1727735587845355</v>
+        <v>0.567670166528999</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>0.08337812122162949</v>
+        <v>0.273950487129699</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>4658031.659165954</v>
+        <v>15304638.88995023</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>1929337.8795</v>
@@ -7515,13 +7515,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>204572003174.7647</v>
+        <v>670725322277.7625</v>
       </c>
       <c r="E21" t="n">
         <v>2653920</v>
       </c>
       <c r="F21" t="n">
-        <v>4976.446993016055</v>
+        <v>16369.4144402207</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -7539,16 +7539,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>4976.446993016055</v>
+        <v>16369.4144402207</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0.1874216627349249</v>
+        <v>0.6165057331643525</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>0.09044810802733161</v>
+        <v>0.2975212368273295</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>5053161.540511617</v>
+        <v>16621969.03072156</v>
       </c>
       <c r="P21" s="4" t="n">
         <v>1663924.6505</v>
@@ -7574,13 +7574,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>38153266139.19757</v>
+        <v>90134099706.92458</v>
       </c>
       <c r="E22" t="n">
         <v>508435.2</v>
       </c>
       <c r="F22" t="n">
-        <v>1067.18566594088</v>
+        <v>2565.276057210292</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -7598,16 +7598,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>1067.18566594088</v>
+        <v>2565.276057210292</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>0.04020751026276068</v>
+        <v>0.09665374264898116</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>0.01941488008134874</v>
+        <v>0.04667233807461426</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>1084563.495719576</v>
+        <v>2607236.909158523</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>689012.1555</v>
@@ -7633,13 +7633,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>39093629028.98856</v>
+        <v>92490994507.14915</v>
       </c>
       <c r="E23" t="n">
         <v>529852.7999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>1252.61724340169</v>
+        <v>3028.972136532676</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -7657,16 +7657,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>1252.61724340169</v>
+        <v>3028.972136532676</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>0.04719745516426868</v>
+        <v>0.1141330137212786</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>0.02278344884494659</v>
+        <v>0.05509588721995031</v>
       </c>
       <c r="O23" s="4" t="n">
-        <v>1272986.377205018</v>
+        <v>3078412.941014688</v>
       </c>
       <c r="P23" s="4" t="n">
         <v>698559.1495000001</v>
@@ -7692,13 +7692,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>38342696728.86106</v>
+        <v>90614396758.013</v>
       </c>
       <c r="E24" t="n">
         <v>515884.8</v>
       </c>
       <c r="F24" t="n">
-        <v>1142.336921530873</v>
+        <v>2753.285671646665</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -7716,16 +7716,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>1142.336921530873</v>
+        <v>2753.285671646665</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>0.0430397659661072</v>
+        <v>0.1037393304550327</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>0.02077703132808371</v>
+        <v>0.05008010384483747</v>
       </c>
       <c r="O24" s="4" t="n">
-        <v>1160821.53924672</v>
+        <v>2798015.393103261</v>
       </c>
       <c r="P24" s="4" t="n">
         <v>690225.7154999999</v>
@@ -7751,13 +7751,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>37834039978.64439</v>
+        <v>89342761464.93727</v>
       </c>
       <c r="E25" t="n">
         <v>506572.8</v>
       </c>
       <c r="F25" t="n">
-        <v>1052.931970048123</v>
+        <v>2529.773421713371</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -7775,16 +7775,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>1052.931970048123</v>
+        <v>2529.773421713371</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>0.03966801424067684</v>
+        <v>0.09530995598830956</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>0.01914863080991969</v>
+        <v>0.0460091048880134</v>
       </c>
       <c r="O25" s="4" t="n">
-        <v>1069824.932926143</v>
+        <v>2570524.007936024</v>
       </c>
       <c r="P25" s="4" t="n">
         <v>675364.0695</v>
@@ -7810,13 +7810,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>38043414109.52127</v>
+        <v>89863478529.43782</v>
       </c>
       <c r="E26" t="n">
         <v>506572.8</v>
       </c>
       <c r="F26" t="n">
-        <v>1054.545046353736</v>
+        <v>2533.752934774764</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -7834,16 +7834,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>1054.545046353736</v>
+        <v>2533.752934774764</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>0.03973860635040877</v>
+        <v>0.09548443473022909</v>
       </c>
       <c r="N26" s="4" t="n">
-        <v>0.01919351789024178</v>
+        <v>0.04612035685787398</v>
       </c>
       <c r="O26" s="4" t="n">
-        <v>1072231.255874496</v>
+        <v>2576485.869249226</v>
       </c>
       <c r="P26" s="4" t="n">
         <v>686420.9135</v>
@@ -7869,13 +7869,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>37359989902.81406</v>
+        <v>88149476858.2751</v>
       </c>
       <c r="E27" t="n">
         <v>492604.8</v>
       </c>
       <c r="F27" t="n">
-        <v>942.4386036831032</v>
+        <v>2253.380382134857</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -7893,16 +7893,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>942.4386036831032</v>
+        <v>2253.380382134857</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>0.03552384399687809</v>
+        <v>0.08494352237307626</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>0.01717808702872767</v>
+        <v>0.04107984659757677</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>960485.5461196182</v>
+        <v>2297013.610876977</v>
       </c>
       <c r="P27" s="4" t="n">
         <v>667391.446</v>
@@ -7928,13 +7928,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>37014631878.12913</v>
+        <v>87293358948.14078</v>
       </c>
       <c r="E28" t="n">
         <v>490742.4</v>
       </c>
       <c r="F28" t="n">
-        <v>950.6146475259378</v>
+        <v>2273.962855540778</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -7952,16 +7952,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>950.6146475259378</v>
+        <v>2273.962855540778</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>0.03581567661713759</v>
+        <v>0.08567846229283269</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>0.0172986853474547</v>
+        <v>0.04138392778491727</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>966298.628697512</v>
+        <v>2311690.738112581</v>
       </c>
       <c r="P28" s="4" t="n">
         <v>650094.7784999999</v>

</xml_diff>

<commit_message>
Update optimization-engineer prompt to handle explicit Pareto rejections (default to single-objective max_profit).
</commit_message>
<xml_diff>
--- a/src/strap/waste_management/Data for model_Scenarios.xlsx
+++ b/src/strap/waste_management/Data for model_Scenarios.xlsx
@@ -6394,13 +6394,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>665218245883.6273</v>
+        <v>202926111011.0003</v>
       </c>
       <c r="E2" t="n">
         <v>2642745.600000001</v>
       </c>
       <c r="F2" t="n">
-        <v>15666.63019162362</v>
+        <v>4765.733611442293</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -6418,16 +6418,16 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>15666.63019162362</v>
+        <v>4765.733611442293</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>0.5901572639578164</v>
+        <v>0.1795217098507607</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>0.2849813592682811</v>
+        <v>0.08668835839130783</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>15918578.82709316</v>
+        <v>4842268.133639095</v>
       </c>
       <c r="P2" s="4" t="n">
         <v>1645223.07</v>
@@ -6453,13 +6453,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>666525829696.7694</v>
+        <v>203322812427.7126</v>
       </c>
       <c r="E3" t="n">
         <v>2642745.600000001</v>
       </c>
       <c r="F3" t="n">
-        <v>15662.39951584713</v>
+        <v>4764.551000420273</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -6477,16 +6477,16 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>15662.39951584713</v>
+        <v>4764.551000420273</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.5900049962128856</v>
+        <v>0.1794792887150163</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.2849159779978077</v>
+        <v>0.08667031655450493</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>15914783.60232515</v>
+        <v>4841217.409068097</v>
       </c>
       <c r="P3" s="4" t="n">
         <v>1649512.153</v>
@@ -6512,13 +6512,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>625232124635.0183</v>
+        <v>190737625701.4836</v>
       </c>
       <c r="E4" t="n">
         <v>2536588.8</v>
       </c>
       <c r="F4" t="n">
-        <v>13455.95924340548</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -6536,16 +6536,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>13455.95924340548</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.5065779354407081</v>
+        <v>0.1543060585272763</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0.2445439553938083</v>
+        <v>0.07448869386639052</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>13656016.62047045</v>
+        <v>4159676.202236705</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>1376265.6805</v>
@@ -6571,13 +6571,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>659926710982.4099</v>
+        <v>201270843091.6686</v>
       </c>
       <c r="E5" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F5" t="n">
-        <v>16057.66494595068</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -6595,16 +6595,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>16057.66494595068</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0.6048612169850395</v>
+        <v>0.1838829672485295</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.2920240650367384</v>
+        <v>0.08877707982610991</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>16314268.07134834</v>
+        <v>4959629.214836514</v>
       </c>
       <c r="P5" s="4" t="n">
         <v>1588570.236</v>
@@ -6630,13 +6630,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>666912636947.7731</v>
+        <v>203478955758.8295</v>
       </c>
       <c r="E6" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F6" t="n">
-        <v>15152.8425063876</v>
+        <v>4612.468401356312</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -6654,16 +6654,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>15152.8425063876</v>
+        <v>4612.468401356312</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>0.570663539923043</v>
+        <v>0.1737063794243001</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>0.2754378429119639</v>
+        <v>0.08384112296942654</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>15388132.66903725</v>
+        <v>4684017.96801324</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>1674069.678</v>
@@ -6689,13 +6689,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>727818948453.0715</v>
+        <v>221770868690.6884</v>
       </c>
       <c r="E7" t="n">
         <v>2866233.6</v>
       </c>
       <c r="F7" t="n">
-        <v>23554.24532157016</v>
+        <v>7133.280889431222</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -6713,16 +6713,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>23554.24532157016</v>
+        <v>7133.280889431222</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.8876410227096855</v>
+        <v>0.2688143651603698</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.4292968209774043</v>
+        <v>0.1300059288112211</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>23969106.23537641</v>
+        <v>7258707.340225391</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>1894036.3775</v>
@@ -6748,13 +6748,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>677213565060.4402</v>
+        <v>206620827403.3771</v>
       </c>
       <c r="E8" t="n">
         <v>2659507.2</v>
       </c>
       <c r="F8" t="n">
-        <v>15568.81932111654</v>
+        <v>4738.270770013095</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -6772,16 +6772,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>15568.81932111654</v>
+        <v>4738.270770013095</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>0.5862860872937612</v>
+        <v>0.1784311331513977</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>0.2829331972787671</v>
+        <v>0.08610805906069278</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>15806838.51117178</v>
+        <v>4810653.628441143</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>1746245.131</v>
@@ -6807,13 +6807,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>659990021842.691</v>
+        <v>201354897959.7589</v>
       </c>
       <c r="E9" t="n">
         <v>2720966.4</v>
       </c>
       <c r="F9" t="n">
-        <v>15074.54702536651</v>
+        <v>4588.054944384647</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -6831,16 +6831,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>15074.54702536651</v>
+        <v>4588.054944384647</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.567670166528999</v>
+        <v>0.1727735587845355</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>0.273950487129699</v>
+        <v>0.08337812122162949</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>15304638.88995023</v>
+        <v>4658031.659165952</v>
       </c>
       <c r="P9" s="4" t="n">
         <v>1935089.606</v>
@@ -6866,13 +6866,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>670725322277.7625</v>
+        <v>204572003174.7647</v>
       </c>
       <c r="E10" t="n">
         <v>2659507.2</v>
       </c>
       <c r="F10" t="n">
-        <v>16369.4144402207</v>
+        <v>4976.446993016055</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -6890,16 +6890,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>16369.4144402207</v>
+        <v>4976.446993016055</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0.6165057331643525</v>
+        <v>0.1874216627349249</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>0.2975212368273295</v>
+        <v>0.09044810802733161</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>16621969.03072156</v>
+        <v>5053161.540511617</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>1661215.79</v>
@@ -6925,13 +6925,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>89342761464.93727</v>
+        <v>37834039978.64438</v>
       </c>
       <c r="E11" t="n">
         <v>616454.4</v>
       </c>
       <c r="F11" t="n">
-        <v>2529.773421713371</v>
+        <v>1052.931970048123</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -6949,16 +6949,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>2529.773421713371</v>
+        <v>1052.931970048123</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.09530995598830956</v>
+        <v>0.03966801424067684</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>0.0460091048880134</v>
+        <v>0.01914863080991969</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>2570524.007936024</v>
+        <v>1069824.932926143</v>
       </c>
       <c r="P11" s="4" t="n">
         <v>827574.618</v>
@@ -6984,13 +6984,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>88149476858.2751</v>
+        <v>37359989902.81407</v>
       </c>
       <c r="E12" t="n">
         <v>586656</v>
       </c>
       <c r="F12" t="n">
-        <v>2253.380382134857</v>
+        <v>942.4386036831032</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -7008,16 +7008,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>2253.380382134857</v>
+        <v>942.4386036831032</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>0.08494352237307626</v>
+        <v>0.03552384399687809</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>0.04107984659757677</v>
+        <v>0.01717808702872767</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2297013.610876977</v>
+        <v>960485.5461196182</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>831337.1199999999</v>
@@ -7043,13 +7043,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>665218245883.6273</v>
+        <v>202926111011.0003</v>
       </c>
       <c r="E13" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F13" t="n">
-        <v>15666.63019162362</v>
+        <v>4765.733611442293</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -7067,16 +7067,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>15666.63019162362</v>
+        <v>4765.733611442293</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0.5901572639578164</v>
+        <v>0.1795217098507607</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.2849813592682811</v>
+        <v>0.08668835839130783</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>15918578.82709316</v>
+        <v>4842268.133639095</v>
       </c>
       <c r="P13" s="4" t="n">
         <v>1640984.363</v>
@@ -7102,13 +7102,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>666525829696.7694</v>
+        <v>203322812427.7126</v>
       </c>
       <c r="E14" t="n">
         <v>2637158.4</v>
       </c>
       <c r="F14" t="n">
-        <v>15662.39951584713</v>
+        <v>4764.551000420273</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -7126,16 +7126,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>15662.39951584713</v>
+        <v>4764.551000420273</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>0.5900049962128856</v>
+        <v>0.1794792887150163</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>0.2849159779978077</v>
+        <v>0.08667031655450493</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>15914783.60232515</v>
+        <v>4841217.409068097</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>1652358.963</v>
@@ -7161,13 +7161,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>625232124635.0183</v>
+        <v>190737625701.4836</v>
       </c>
       <c r="E15" t="n">
         <v>2536588.8</v>
       </c>
       <c r="F15" t="n">
-        <v>13455.95924340548</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -7185,16 +7185,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>13455.95924340548</v>
+        <v>4098.763512502049</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.5065779354407081</v>
+        <v>0.1543060585272763</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.2445439553938083</v>
+        <v>0.07448869386639052</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>13656016.62047045</v>
+        <v>4159676.202236705</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>1371700.307</v>
@@ -7220,13 +7220,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>659926710982.4099</v>
+        <v>201270843091.6686</v>
       </c>
       <c r="E16" t="n">
         <v>2631571.2</v>
       </c>
       <c r="F16" t="n">
-        <v>16057.66494595068</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -7244,16 +7244,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>16057.66494595068</v>
+        <v>4881.717512393886</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>0.6048612169850395</v>
+        <v>0.1838829672485295</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>0.2920240650367384</v>
+        <v>0.08877707982610991</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>16314268.07134834</v>
+        <v>4959629.214836514</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>1590719.481</v>
@@ -7279,13 +7279,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>666912636947.7731</v>
+        <v>203478955758.8295</v>
       </c>
       <c r="E17" t="n">
         <v>2631571.2</v>
       </c>
       <c r="F17" t="n">
-        <v>15152.8425063876</v>
+        <v>4612.468401356312</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -7303,16 +7303,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>15152.8425063876</v>
+        <v>4612.468401356312</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.570663539923043</v>
+        <v>0.1737063794243001</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>0.2754378429119639</v>
+        <v>0.08384112296942654</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>15388132.66903725</v>
+        <v>4684017.96801324</v>
       </c>
       <c r="P17" s="4" t="n">
         <v>1670234.7225</v>
@@ -7338,13 +7338,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>727818948453.0715</v>
+        <v>221770868690.6884</v>
       </c>
       <c r="E18" t="n">
         <v>2855059.2</v>
       </c>
       <c r="F18" t="n">
-        <v>23554.24532157016</v>
+        <v>7133.280889431222</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -7362,16 +7362,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>23554.24532157016</v>
+        <v>7133.280889431222</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0.8876410227096855</v>
+        <v>0.2688143651603698</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>0.4292968209774043</v>
+        <v>0.1300059288112211</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>23969106.23537641</v>
+        <v>7258707.340225391</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>1893805.082</v>
@@ -7397,13 +7397,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>677213565060.4402</v>
+        <v>206620827403.3771</v>
       </c>
       <c r="E19" t="n">
         <v>2653920</v>
       </c>
       <c r="F19" t="n">
-        <v>15568.81932111654</v>
+        <v>4738.270770013095</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -7421,16 +7421,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>15568.81932111654</v>
+        <v>4738.270770013095</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>0.5862860872937612</v>
+        <v>0.1784311331513977</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>0.2829331972787671</v>
+        <v>0.08610805906069278</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>15806838.51117178</v>
+        <v>4810653.628441143</v>
       </c>
       <c r="P19" s="4" t="n">
         <v>1742565.4565</v>
@@ -7456,13 +7456,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>659990021842.691</v>
+        <v>201354897959.7589</v>
       </c>
       <c r="E20" t="n">
         <v>2715379.2</v>
       </c>
       <c r="F20" t="n">
-        <v>15074.54702536651</v>
+        <v>4588.054944384647</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -7480,16 +7480,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>15074.54702536651</v>
+        <v>4588.054944384647</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>0.567670166528999</v>
+        <v>0.1727735587845355</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>0.273950487129699</v>
+        <v>0.08337812122162949</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>15304638.88995023</v>
+        <v>4658031.659165952</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>1929337.8795</v>
@@ -7515,13 +7515,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>670725322277.7625</v>
+        <v>204572003174.7647</v>
       </c>
       <c r="E21" t="n">
         <v>2653920</v>
       </c>
       <c r="F21" t="n">
-        <v>16369.4144402207</v>
+        <v>4976.446993016055</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -7539,16 +7539,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>16369.4144402207</v>
+        <v>4976.446993016055</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0.6165057331643525</v>
+        <v>0.1874216627349249</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>0.2975212368273295</v>
+        <v>0.09044810802733161</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>16621969.03072156</v>
+        <v>5053161.540511617</v>
       </c>
       <c r="P21" s="4" t="n">
         <v>1663924.6505</v>
@@ -7574,13 +7574,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>90134099706.92458</v>
+        <v>38153266139.19757</v>
       </c>
       <c r="E22" t="n">
         <v>508435.2</v>
       </c>
       <c r="F22" t="n">
-        <v>2565.276057210292</v>
+        <v>1067.18566594088</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -7598,16 +7598,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>2565.276057210292</v>
+        <v>1067.18566594088</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>0.09665374264898116</v>
+        <v>0.04020751026276068</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>0.04667233807461426</v>
+        <v>0.01941488008134874</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>2607236.909158523</v>
+        <v>1084563.495719576</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>689012.1555</v>
@@ -7633,13 +7633,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>92490994507.14915</v>
+        <v>39093629028.98856</v>
       </c>
       <c r="E23" t="n">
         <v>529852.7999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>3028.972136532676</v>
+        <v>1252.61724340169</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -7657,16 +7657,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>3028.972136532676</v>
+        <v>1252.61724340169</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>0.1141330137212786</v>
+        <v>0.04719745516426868</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>0.05509588721995031</v>
+        <v>0.02278344884494659</v>
       </c>
       <c r="O23" s="4" t="n">
-        <v>3078412.941014688</v>
+        <v>1272986.377205018</v>
       </c>
       <c r="P23" s="4" t="n">
         <v>698559.1495000001</v>
@@ -7692,13 +7692,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>90614396758.013</v>
+        <v>38342696728.86106</v>
       </c>
       <c r="E24" t="n">
         <v>515884.8</v>
       </c>
       <c r="F24" t="n">
-        <v>2753.285671646665</v>
+        <v>1142.336921530873</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -7716,16 +7716,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>2753.285671646665</v>
+        <v>1142.336921530873</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>0.1037393304550327</v>
+        <v>0.04303976596610721</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>0.05008010384483747</v>
+        <v>0.02077703132808372</v>
       </c>
       <c r="O24" s="4" t="n">
-        <v>2798015.393103261</v>
+        <v>1160821.53924672</v>
       </c>
       <c r="P24" s="4" t="n">
         <v>690225.7154999999</v>
@@ -7751,13 +7751,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>89342761464.93727</v>
+        <v>37834039978.64438</v>
       </c>
       <c r="E25" t="n">
         <v>506572.8</v>
       </c>
       <c r="F25" t="n">
-        <v>2529.773421713371</v>
+        <v>1052.931970048123</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -7775,16 +7775,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>2529.773421713371</v>
+        <v>1052.931970048123</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>0.09530995598830956</v>
+        <v>0.03966801424067684</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>0.0460091048880134</v>
+        <v>0.01914863080991969</v>
       </c>
       <c r="O25" s="4" t="n">
-        <v>2570524.007936024</v>
+        <v>1069824.932926143</v>
       </c>
       <c r="P25" s="4" t="n">
         <v>675364.0695</v>
@@ -7810,13 +7810,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>89863478529.43782</v>
+        <v>38043414109.52127</v>
       </c>
       <c r="E26" t="n">
         <v>506572.8</v>
       </c>
       <c r="F26" t="n">
-        <v>2533.752934774764</v>
+        <v>1054.545046353736</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -7834,16 +7834,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>2533.752934774764</v>
+        <v>1054.545046353736</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>0.09548443473022909</v>
+        <v>0.03973860635040877</v>
       </c>
       <c r="N26" s="4" t="n">
-        <v>0.04612035685787398</v>
+        <v>0.01919351789024178</v>
       </c>
       <c r="O26" s="4" t="n">
-        <v>2576485.869249226</v>
+        <v>1072231.255874496</v>
       </c>
       <c r="P26" s="4" t="n">
         <v>686420.9135</v>
@@ -7869,13 +7869,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>88149476858.2751</v>
+        <v>37359989902.81407</v>
       </c>
       <c r="E27" t="n">
         <v>492604.8</v>
       </c>
       <c r="F27" t="n">
-        <v>2253.380382134857</v>
+        <v>942.4386036831032</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -7893,16 +7893,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>2253.380382134857</v>
+        <v>942.4386036831032</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>0.08494352237307626</v>
+        <v>0.03552384399687809</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>0.04107984659757677</v>
+        <v>0.01717808702872767</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>2297013.610876977</v>
+        <v>960485.5461196182</v>
       </c>
       <c r="P27" s="4" t="n">
         <v>667391.446</v>
@@ -7928,13 +7928,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>87293358948.14078</v>
+        <v>37014631878.12914</v>
       </c>
       <c r="E28" t="n">
         <v>490742.4</v>
       </c>
       <c r="F28" t="n">
-        <v>2273.962855540778</v>
+        <v>950.6146475259378</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -7952,16 +7952,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>2273.962855540778</v>
+        <v>950.6146475259378</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>0.08567846229283269</v>
+        <v>0.03581567661713759</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>0.04138392778491727</v>
+        <v>0.0172986853474547</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>2311690.738112581</v>
+        <v>966298.628697512</v>
       </c>
       <c r="P28" s="4" t="n">
         <v>650094.7784999999</v>

</xml_diff>